<commit_message>
Added consultor to sentinela and consulta
</commit_message>
<xml_diff>
--- a/app/config/tables/sentinela/forms/consulta/consulta.xlsx
+++ b/app/config/tables/sentinela/forms/consulta/consulta.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0" codeName="ThisWorkbook" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\celso\ODKX\app-designer\app\config\tables\sentinela\forms\consulta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\celso\odkx\sentinela\app\config\tables\sentinela\forms\consulta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CADE8BDA-5EB5-4CF1-9F00-3E02F42DB26E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56B88FA0-FA29-4B72-AE01-E5A8782D0B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="3" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="222">
   <si>
     <t>type</t>
   </si>
@@ -697,6 +697,9 @@
   </si>
   <si>
     <t>Centro: {{data('csname')}} Data: {{calculates.hoje_display}}</t>
+  </si>
+  <si>
+    <t>consultor</t>
   </si>
 </sst>
 </file>
@@ -3486,7 +3489,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultColWidth="11.5" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.125" customWidth="1"/>
@@ -3675,6 +3678,14 @@
       </c>
       <c r="B23" s="10" t="s">
         <v>219</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reverted xlsx to match x.sapiens
</commit_message>
<xml_diff>
--- a/app/config/tables/sentinela/forms/consulta/consulta.xlsx
+++ b/app/config/tables/sentinela/forms/consulta/consulta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\celso\odkx\sentinela\app\config\tables\sentinela\forms\consulta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B601285B-BD1E-47B7-B2A2-15E31B3421A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E22FCAF-874C-4DBB-AEBB-27E461949679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,15 +24,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">survey!$D$1:$K$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
     </ext>
@@ -118,6 +111,9 @@
     <t>sexo</t>
   </si>
   <si>
+    <t>Sexo</t>
+  </si>
+  <si>
     <t>Data de Nascimento</t>
   </si>
   <si>
@@ -646,6 +642,9 @@
     <t>select_one_dropdown</t>
   </si>
   <si>
+    <t>data('sexo')=='2' &amp;&amp; (calculates.idade_mes()&lt;=660 &amp;&amp; calculates.idade_mes()&gt;=144)</t>
+  </si>
+  <si>
     <t>comentario</t>
   </si>
   <si>
@@ -685,28 +684,22 @@
     <t>csname</t>
   </si>
   <si>
+    <t>Centro: {{data.csname}} Data: {{calculates.hoje_display}}</t>
+  </si>
+  <si>
     <t>consultor</t>
   </si>
   <si>
+    <t>data('DOB_idade')=='1' ? adate.ageInMonths(data('dn')) : 12 * parseInt(data('ano'),10)</t>
+  </si>
+  <si>
+    <t>child_adult</t>
+  </si>
+  <si>
+    <t>data('cs') + calculates.child_adult()</t>
+  </si>
+  <si>
     <t>Proveniência</t>
-  </si>
-  <si>
-    <t>child_adult</t>
-  </si>
-  <si>
-    <t>data('cs') + calculates.child_adult()</t>
-  </si>
-  <si>
-    <t>data('sexo')=='2' &amp;&amp; calculates.idade_mes() &gt;= 144 &amp;&amp; calculates.idade_mes() &lt;= 660</t>
-  </si>
-  <si>
-    <t>Sexo</t>
-  </si>
-  <si>
-    <t>data('DOB_idade')=='1' ? adate.ageInMonths(data('dn')) : 12 * parseInt(data('ano'),10)</t>
-  </si>
-  <si>
-    <t>Centro: {{data.csname}} Data: {{calculates.hoje_display}}</t>
   </si>
 </sst>
 </file>
@@ -1346,7 +1339,7 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1362,7 +1355,7 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1370,15 +1363,15 @@
         <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1417,7 +1410,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>8</v>
@@ -1438,7 +1431,7 @@
         <v>20</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I1" t="s">
         <v>21</v>
@@ -1453,37 +1446,37 @@
         <v>3</v>
       </c>
       <c r="M1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O1" s="20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="P1" s="20" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="R1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="T1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="U1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="V1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="W1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X1" t="s">
         <v>19</v>
@@ -1524,20 +1517,20 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="D6" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J6" s="24"/>
       <c r="K6" s="2"/>
       <c r="N6" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="R6"/>
       <c r="S6"/>
@@ -1547,13 +1540,13 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="D7" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="J7" s="25"/>
       <c r="K7" s="2"/>
@@ -1566,13 +1559,13 @@
         <v>10</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L8" s="2" t="b">
         <v>1</v>
@@ -1580,10 +1573,10 @@
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E9" s="12"/>
       <c r="F9" s="12"/>
@@ -1592,22 +1585,22 @@
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="C10" s="12"/>
       <c r="D10" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E10" s="12"/>
       <c r="F10" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="G10" s="12" t="s">
-        <v>25</v>
-      </c>
       <c r="L10" s="11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="11"/>
       <c r="E11" s="12"/>
@@ -1620,24 +1613,24 @@
       </c>
       <c r="E12" s="12"/>
       <c r="F12" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="L12" s="11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E13" s="12"/>
       <c r="F13" s="12"/>
@@ -1650,29 +1643,29 @@
       </c>
       <c r="E14" s="12"/>
       <c r="F14" s="12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I14" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="J14" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="L14" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C17" s="11"/>
       <c r="E17" s="12"/>
@@ -1680,7 +1673,7 @@
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C18" s="11"/>
       <c r="E18" s="12"/>
@@ -1693,7 +1686,7 @@
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="10"/>
@@ -1713,10 +1706,10 @@
       </c>
       <c r="E21" s="9"/>
       <c r="F21" s="10" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
@@ -1729,14 +1722,14 @@
     <row r="22" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C22" s="11"/>
       <c r="D22" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E22" s="12"/>
       <c r="F22" s="12" t="s">
         <v>23</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="L22" s="2" t="b">
         <v>1</v>
@@ -1745,14 +1738,14 @@
     <row r="23" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C23" s="11"/>
       <c r="D23" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E23" s="12"/>
       <c r="F23" s="12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -1767,7 +1760,7 @@
         <v>24</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>219</v>
+        <v>25</v>
       </c>
       <c r="L24" s="2" t="b">
         <v>1</v>
@@ -1775,10 +1768,10 @@
     </row>
     <row r="25" spans="2:14" ht="47.25" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>218</v>
+        <v>202</v>
       </c>
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.25">
@@ -1786,23 +1779,23 @@
         <v>10</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B27" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C28" s="11"/>
       <c r="E28" s="12"/>
@@ -1811,14 +1804,14 @@
     <row r="29" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C29" s="11"/>
       <c r="D29" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E29" s="13"/>
       <c r="F29" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N29" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.25">
@@ -1828,34 +1821,34 @@
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B31" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.25">
       <c r="D32" s="12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="C33" s="11"/>
       <c r="D33" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E33"/>
       <c r="F33" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G33" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.25">
@@ -1864,59 +1857,59 @@
         <v>10</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="35" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
       <c r="C35" s="11"/>
       <c r="D35" s="12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E35" s="12"/>
       <c r="F35" s="12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="C36" s="12"/>
       <c r="D36" s="12" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="C37" s="11"/>
       <c r="D37" s="12" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.25">
@@ -1924,13 +1917,13 @@
         <v>10</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J38" s="7"/>
       <c r="K38" s="2"/>
@@ -1939,7 +1932,7 @@
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B39" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C39" s="11"/>
       <c r="E39" s="12"/>
@@ -1948,7 +1941,7 @@
     <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A40"/>
       <c r="B40" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C40" s="11"/>
       <c r="E40" s="12"/>
@@ -1956,27 +1949,27 @@
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="D41" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42"/>
       <c r="D42" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B43" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.25">
@@ -1984,10 +1977,10 @@
         <v>4</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.25">
@@ -2391,7 +2384,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2402,29 +2395,29 @@
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B5" s="2">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B6" s="2">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -2433,24 +2426,24 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B8" s="2">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -2459,101 +2452,101 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B11" s="2">
         <v>1</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B12" s="2">
         <v>2</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B13" s="2">
         <v>3</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B14" s="2">
         <v>4</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>195</v>
-      </c>
       <c r="C19" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -2561,332 +2554,332 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -3285,63 +3278,63 @@
   <sheetData>
     <row r="1" spans="1:11" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="C1" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="G1" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="H1" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="I1" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="J1" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" s="23" t="s">
-        <v>72</v>
-      </c>
-      <c r="E1" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="F1" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="G1" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="H1" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="I1" s="23" t="s">
-        <v>77</v>
-      </c>
-      <c r="J1" s="23" t="s">
+      <c r="K1" s="23" t="s">
         <v>40</v>
-      </c>
-      <c r="K1" s="23" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="G2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="H2" s="22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -3366,44 +3359,44 @@
   <sheetData>
     <row r="1" spans="1:4" s="21" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B1" s="20" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D1" s="20" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -3422,50 +3415,50 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" t="s">
         <v>87</v>
-      </c>
-      <c r="B2" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B4" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B6" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -3513,10 +3506,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3524,7 +3517,7 @@
         <v>10</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3532,15 +3525,15 @@
         <v>10</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3548,7 +3541,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3556,20 +3549,20 @@
         <v>5</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>23</v>
@@ -3577,10 +3570,10 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3596,23 +3589,23 @@
         <v>10</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3620,31 +3613,31 @@
         <v>10</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3652,7 +3645,7 @@
         <v>10</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3660,15 +3653,15 @@
         <v>4</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -3676,23 +3669,23 @@
         <v>5</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>214</v>
+      <c r="A24" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
teste de dia 28/2
</commit_message>
<xml_diff>
--- a/app/config/tables/sentinela/forms/consulta/consulta.xlsx
+++ b/app/config/tables/sentinela/forms/consulta/consulta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\celso\odkx\sentinela\app\config\tables\sentinela\forms\consulta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0FDFFA9-A774-48A4-B78D-7C4DA4287404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6D6E9BF-EADD-49BE-A383-B3423F59167B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="3" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="203">
   <si>
     <t>type</t>
   </si>
@@ -569,6 +569,90 @@
   </si>
   <si>
     <t>["1B75", "MA01", "PJ20", "4A8Z", "JA40_0", "CA23", "CA20", "CA07", "CA20_Y", "CA40_Z", "CA41", "CA00", "1F23_0", "1F23_10", "MD81_4", "EB7Y", "1A40_Z", "GA34_3", "1A40_Z", "DA01", "1G04", "1A07_Z", "1A7Z", "BA00_Z", "BA2Z", "JA60_Z", "AAZ1_90", "1A36_0Z", "1B7Y", "1F03", "MG26", "1B1Z", "DA60", "GC02", "1A92", "1E90", "1C62_Z", "outro"].indexOf(data('diagnostico'))&lt;0 ? 1 : 0</t>
+  </si>
+  <si>
+    <t>Coartem</t>
+  </si>
+  <si>
+    <t>Quinino comp.</t>
+  </si>
+  <si>
+    <t>Quinina injet</t>
+  </si>
+  <si>
+    <t>Artusunato injet</t>
+  </si>
+  <si>
+    <t>tto</t>
+  </si>
+  <si>
+    <t>Outros</t>
+  </si>
+  <si>
+    <t>6/6h</t>
+  </si>
+  <si>
+    <t>8/8h</t>
+  </si>
+  <si>
+    <t>12/12h</t>
+  </si>
+  <si>
+    <t>freq</t>
+  </si>
+  <si>
+    <t>24/24h ou uma vez por dia</t>
+  </si>
+  <si>
+    <t>Oral</t>
+  </si>
+  <si>
+    <t>Intra Venosa</t>
+  </si>
+  <si>
+    <t>vo</t>
+  </si>
+  <si>
+    <t>vm</t>
+  </si>
+  <si>
+    <t>vi</t>
+  </si>
+  <si>
+    <t>via</t>
+  </si>
+  <si>
+    <t>Intra Muscular</t>
+  </si>
+  <si>
+    <t>dose/Kg</t>
+  </si>
+  <si>
+    <t>dose/ml</t>
+  </si>
+  <si>
+    <t>doses</t>
+  </si>
+  <si>
+    <t>Medicamento</t>
+  </si>
+  <si>
+    <t>quanti</t>
+  </si>
+  <si>
+    <t>Doses</t>
+  </si>
+  <si>
+    <t>unidade</t>
+  </si>
+  <si>
+    <t>Unidade de medida de dosis</t>
+  </si>
+  <si>
+    <t>Frequência</t>
+  </si>
+  <si>
+    <t>Via de Administração</t>
   </si>
 </sst>
 </file>
@@ -1782,69 +1866,101 @@
         <v>100</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="C44" s="11"/>
-      <c r="D44" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="E44" s="13"/>
-      <c r="F44" s="12" t="s">
-        <v>157</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="D45" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="F45" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>74</v>
+      <c r="B45" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="B46" s="2" t="s">
-        <v>51</v>
-      </c>
       <c r="C46" s="11"/>
       <c r="E46" s="12"/>
       <c r="F46" s="12"/>
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B47" s="2" t="s">
+        <v>50</v>
+      </c>
       <c r="C47" s="11"/>
       <c r="E47" s="13"/>
       <c r="F47" s="12"/>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C48" s="11"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="12"/>
+      <c r="D48" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E48" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="F48" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="49" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C49" s="11"/>
+      <c r="D49" s="12" t="s">
+        <v>90</v>
+      </c>
       <c r="E49" s="13"/>
-      <c r="F49" s="12"/>
+      <c r="F49" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="50" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C50" s="11"/>
-      <c r="E50" s="13"/>
-      <c r="F50" s="12"/>
+      <c r="D50" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E50" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="F50" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="51" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C51" s="12"/>
-      <c r="E51" s="13"/>
-      <c r="F51" s="12"/>
+      <c r="D51" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E51" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="F51" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="52" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C52" s="11"/>
-      <c r="E52" s="12"/>
-      <c r="F52" s="12"/>
+      <c r="D52" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E52" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="F52" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="53" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B53" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="C53" s="11"/>
       <c r="E53" s="12"/>
       <c r="F53" s="12"/>
@@ -1867,7 +1983,9 @@
       <c r="J55" s="6"/>
     </row>
     <row r="56" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B56" s="13"/>
+      <c r="B56" s="13" t="s">
+        <v>50</v>
+      </c>
       <c r="C56" s="13"/>
       <c r="D56" s="15"/>
       <c r="E56" s="13"/>
@@ -1876,20 +1994,28 @@
       <c r="J56" s="6"/>
     </row>
     <row r="57" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B57" s="13"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="15"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="12" t="s">
+        <v>58</v>
+      </c>
       <c r="E57" s="13"/>
-      <c r="F57" s="16"/>
-      <c r="G57" s="13"/>
+      <c r="F57" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="58" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B58" s="13"/>
-      <c r="C58" s="13"/>
-      <c r="D58" s="15"/>
-      <c r="E58" s="13"/>
-      <c r="F58" s="16"/>
-      <c r="G58" s="13"/>
+      <c r="D58" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="F58" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="59" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B59" s="13"/>
@@ -1900,7 +2026,9 @@
       <c r="G59" s="13"/>
     </row>
     <row r="60" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B60" s="13"/>
+      <c r="B60" s="13" t="s">
+        <v>51</v>
+      </c>
       <c r="C60" s="13"/>
       <c r="D60" s="15"/>
       <c r="E60" s="13"/>
@@ -2424,63 +2552,169 @@
       <c r="A29" s="1"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="1"/>
-      <c r="C30" s="1"/>
+      <c r="A30" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B30" s="2">
+        <v>1</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="1"/>
-      <c r="C31" s="1"/>
+      <c r="A31" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B31" s="2">
+        <v>2</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="1"/>
-      <c r="C32" s="1"/>
+      <c r="A32" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B32" s="2">
+        <v>3</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="1"/>
-      <c r="C33" s="1"/>
+      <c r="A33" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B33" s="2">
+        <v>4</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="1"/>
-      <c r="C34" s="1"/>
+      <c r="A34" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B34" s="2">
+        <v>5</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="C35" s="1"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="1"/>
-      <c r="C36" s="1"/>
+      <c r="A36" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B36" s="2">
+        <v>4</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="1"/>
-      <c r="C37" s="1"/>
+      <c r="A37" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B37" s="2">
+        <v>3</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>182</v>
+      </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="1"/>
-      <c r="C38" s="1"/>
+      <c r="A38" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B38" s="2">
+        <v>2</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="1"/>
-      <c r="C39" s="1"/>
+      <c r="A39" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B39" s="2">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="C40" s="1"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="1"/>
-      <c r="C41" s="1"/>
+      <c r="A41" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="1"/>
-      <c r="C42" s="1"/>
+      <c r="A42" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="1"/>
-      <c r="C43" s="1"/>
+      <c r="A43" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B45" s="2">
+        <v>1</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B46" s="2">
+        <v>2</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" s="1"/>
@@ -2854,7 +3088,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr defaultColWidth="11.5" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.125" customWidth="1"/>
@@ -3111,6 +3345,46 @@
       </c>
       <c r="B35" s="2" t="s">
         <v>145</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed stupid odk-x bug with blank lines
</commit_message>
<xml_diff>
--- a/app/config/tables/sentinela/forms/consulta/consulta.xlsx
+++ b/app/config/tables/sentinela/forms/consulta/consulta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\celso\odkx\sentinela\app\config\tables\sentinela\forms\consulta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FBE6243-D2C5-4D08-8A44-C2154EDB6A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE50E8F1-FC1F-49CC-9BE5-837AC76074B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-285" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="3" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="200">
   <si>
     <t>type</t>
   </si>
@@ -768,21 +768,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1342,19 +1333,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:Z94"/>
+  <dimension ref="A1:Z84"/>
   <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.875" style="2" customWidth="1"/>
     <col min="2" max="2" width="12.25" style="2" customWidth="1"/>
     <col min="3" max="3" width="94.75" style="2" customWidth="1"/>
-    <col min="4" max="4" width="25.375" style="12" customWidth="1"/>
+    <col min="4" max="4" width="25.375" style="9" customWidth="1"/>
     <col min="5" max="5" width="16.125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="17.5" style="11" customWidth="1"/>
+    <col min="6" max="6" width="17.5" style="8" customWidth="1"/>
     <col min="7" max="7" width="63" style="2" customWidth="1"/>
     <col min="8" max="8" width="29.75" style="2" customWidth="1"/>
     <col min="9" max="9" width="24.125" style="2" customWidth="1"/>
-    <col min="10" max="10" width="10.75" style="7"/>
+    <col min="10" max="10" width="10.75" style="4"/>
     <col min="11" max="11" width="28.5" style="2" customWidth="1"/>
     <col min="12" max="12" width="13.25" style="2" customWidth="1"/>
     <col min="13" max="13" width="17" style="2" customWidth="1"/>
@@ -1374,13 +1365,13 @@
       <c r="C1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="8" t="s">
         <v>1</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -1410,10 +1401,10 @@
       <c r="O1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="P1" s="19" t="s">
+      <c r="P1" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="Q1" s="19" t="s">
+      <c r="Q1" s="16" t="s">
         <v>81</v>
       </c>
       <c r="R1" t="s">
@@ -1445,779 +1436,714 @@
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="4"/>
-    </row>
-    <row r="3" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="4"/>
-    </row>
-    <row r="4" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="4"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E2" s="20"/>
+      <c r="F2" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="N2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="D4" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="C5" s="11"/>
-      <c r="D5" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E5" s="23"/>
-      <c r="F5" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="N5" t="s">
-        <v>126</v>
+      <c r="B5" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="B6" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="5"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="K6" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>120</v>
-      </c>
+      <c r="C7" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="D8" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>87</v>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9" t="s">
+        <v>135</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>88</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="L8" s="9"/>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>52</v>
       </c>
+      <c r="C9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="C10" s="11"/>
-      <c r="D10" s="9"/>
-      <c r="E10"/>
-      <c r="F10" s="17"/>
-      <c r="G10"/>
+      <c r="C10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="B11" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+    </row>
+    <row r="12" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="9"/>
+      <c r="D12" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="O12" s="2" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="9"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="9"/>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="C14" s="9"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="9"/>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="C15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="C16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+    </row>
+    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C18" s="8"/>
+      <c r="D18" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C19" s="8"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+    </row>
+    <row r="21" spans="2:20" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C21" s="9"/>
+      <c r="D21" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="K21" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="L21" s="9"/>
+    </row>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+    </row>
+    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+    </row>
+    <row r="24" spans="2:20" ht="63" x14ac:dyDescent="0.25">
+      <c r="B24" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+    </row>
+    <row r="25" spans="2:20" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C25" s="9"/>
+      <c r="D25" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="J25" s="28"/>
+      <c r="O25" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="P25" s="14"/>
+      <c r="Q25" s="14"/>
+    </row>
+    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B26" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="9"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="9"/>
+    </row>
+    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C27" s="9"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="9"/>
+    </row>
+    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="C28" s="9"/>
+      <c r="D28" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="29" spans="2:20" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29" s="24" t="s">
+        <v>196</v>
+      </c>
+      <c r="D29" s="24"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="24"/>
+      <c r="J29" s="26"/>
+      <c r="P29" s="27"/>
+      <c r="Q29" s="27"/>
+    </row>
+    <row r="30" spans="2:20" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D30" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E30" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="F30" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="G30" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="I30" s="26"/>
+      <c r="P30" s="27"/>
+      <c r="Q30" s="27"/>
+      <c r="S30" s="27"/>
+      <c r="T30" s="27"/>
+    </row>
+    <row r="31" spans="2:20" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="I31" s="26"/>
+      <c r="P31" s="27"/>
+      <c r="Q31" s="27"/>
+      <c r="S31" s="27"/>
+      <c r="T31" s="27"/>
+    </row>
+    <row r="32" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B32" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C32" s="8"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="9"/>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C33" s="8"/>
+      <c r="D33" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C34" s="8"/>
+      <c r="D34" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="E34" s="10"/>
+      <c r="F34" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C35" s="8"/>
+      <c r="D35" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C36" s="9"/>
+      <c r="D36" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C37" s="8"/>
+      <c r="D37" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B38" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-    </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="C14" s="11"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="C15" s="11"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="C16" s="12"/>
-      <c r="D16" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="K16" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-    </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="C18" s="12"/>
-      <c r="D18" s="12" t="s">
+      <c r="C38" s="8"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="10"/>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B40" s="10"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="12"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="13"/>
+      <c r="G40" s="10"/>
+      <c r="J40" s="3"/>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B41" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C41" s="10"/>
+      <c r="D41" s="12"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="10"/>
+      <c r="J41" s="3"/>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C42" s="8"/>
+      <c r="D42" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="K18" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="L18" s="12"/>
-    </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B19" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-    </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="C20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B21" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-    </row>
-    <row r="22" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C22" s="12"/>
-      <c r="D22" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="F22" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="O22" s="2" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B23" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C23" s="12"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="12"/>
-    </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="C24" s="12"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="12"/>
-    </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="C25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="C26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-    </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="C27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-    </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="C28" s="11"/>
-      <c r="D28" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E28" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="F28" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="C29" s="11"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-    </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B30" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
-    </row>
-    <row r="31" spans="2:15" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="C31" s="12"/>
-      <c r="D31" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="K31" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="L31" s="12"/>
-    </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B32" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C32" s="12"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
-    </row>
-    <row r="33" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="C33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-    </row>
-    <row r="34" spans="2:20" ht="63" x14ac:dyDescent="0.25">
-      <c r="B34" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>198</v>
-      </c>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-    </row>
-    <row r="35" spans="2:20" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C35" s="12"/>
-      <c r="D35" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="F35" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="G35" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="J35" s="31"/>
-      <c r="O35" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="P35" s="17"/>
-      <c r="Q35" s="17"/>
-    </row>
-    <row r="36" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B36" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C36" s="12"/>
-      <c r="E36" s="1"/>
-      <c r="F36" s="12"/>
-    </row>
-    <row r="37" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="C37" s="12"/>
-      <c r="E37" s="1"/>
-      <c r="F37" s="12"/>
-    </row>
-    <row r="38" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="C38" s="12"/>
-      <c r="D38" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F38" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="39" spans="2:20" s="26" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="C39" s="27" t="s">
-        <v>196</v>
-      </c>
-      <c r="D39" s="27"/>
-      <c r="E39" s="28"/>
-      <c r="F39" s="27"/>
-      <c r="J39" s="29"/>
-      <c r="P39" s="30"/>
-      <c r="Q39" s="30"/>
-    </row>
-    <row r="40" spans="2:20" s="26" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D40" s="26" t="s">
-        <v>197</v>
-      </c>
-      <c r="E40" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="F40" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="G40" s="26" t="s">
-        <v>165</v>
-      </c>
-      <c r="I40" s="29"/>
-      <c r="P40" s="30"/>
-      <c r="Q40" s="30"/>
-      <c r="S40" s="30"/>
-      <c r="T40" s="30"/>
-    </row>
-    <row r="41" spans="2:20" s="26" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="I41" s="29"/>
-      <c r="P41" s="30"/>
-      <c r="Q41" s="30"/>
-      <c r="S41" s="30"/>
-      <c r="T41" s="30"/>
-    </row>
-    <row r="42" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B42" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C42" s="11"/>
-      <c r="E42" s="13"/>
-      <c r="F42" s="12"/>
-    </row>
-    <row r="43" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="C43" s="11"/>
-      <c r="D43" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="E43" s="13" t="s">
-        <v>170</v>
-      </c>
-      <c r="F43" s="12" t="s">
-        <v>170</v>
+      <c r="E42" s="10"/>
+      <c r="F42" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D43" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F43" s="8" t="s">
+        <v>121</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="44" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="C44" s="11"/>
-      <c r="D44" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="E44" s="13"/>
-      <c r="F44" s="12" t="s">
-        <v>188</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="45" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="C45" s="11"/>
-      <c r="D45" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="E45" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="F45" s="12" t="s">
-        <v>190</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="46" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="C46" s="12"/>
-      <c r="D46" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="E46" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="F46" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="47" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="C47" s="11"/>
-      <c r="D47" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E47" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="F47" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="48" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B48" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="12"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="10"/>
+    </row>
+    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B45" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C48" s="11"/>
-      <c r="E48" s="12"/>
-      <c r="F48" s="12"/>
-    </row>
-    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B49" s="13"/>
-      <c r="C49" s="13"/>
-      <c r="D49" s="15"/>
-      <c r="E49" s="13"/>
-      <c r="F49" s="16"/>
-      <c r="G49" s="13"/>
-    </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B50" s="13"/>
-      <c r="C50" s="13"/>
-      <c r="D50" s="15"/>
-      <c r="E50" s="13"/>
-      <c r="F50" s="16"/>
-      <c r="G50" s="13"/>
-      <c r="J50" s="6"/>
-    </row>
-    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B51" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="C51" s="13"/>
-      <c r="D51" s="15"/>
-      <c r="E51" s="13"/>
-      <c r="F51" s="16"/>
-      <c r="G51" s="13"/>
-      <c r="J51" s="6"/>
-    </row>
-    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="C52" s="11"/>
-      <c r="D52" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="E52" s="13"/>
-      <c r="F52" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="D53" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="F53" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B54" s="13"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="13"/>
-      <c r="F54" s="16"/>
-      <c r="G54" s="13"/>
-    </row>
-    <row r="55" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B55" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C55" s="13"/>
-      <c r="D55" s="15"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="16"/>
-      <c r="G55" s="13"/>
-    </row>
-    <row r="56" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B56" s="13"/>
-      <c r="C56" s="13"/>
-      <c r="D56" s="15"/>
-      <c r="E56" s="13"/>
-      <c r="F56" s="16"/>
-      <c r="G56" s="13"/>
-    </row>
-    <row r="57" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B57" s="24"/>
-      <c r="C57" s="24"/>
-      <c r="D57" s="25"/>
-      <c r="E57" s="24"/>
-      <c r="F57" s="25"/>
-      <c r="G57" s="24"/>
-    </row>
-    <row r="58" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B58" s="24"/>
-      <c r="C58" s="24"/>
-      <c r="D58" s="25"/>
-      <c r="E58" s="24"/>
-      <c r="F58" s="25"/>
-      <c r="G58" s="24"/>
-    </row>
-    <row r="59" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B59" s="13"/>
-      <c r="C59" s="13"/>
-      <c r="D59" s="15"/>
-      <c r="E59" s="13"/>
-      <c r="F59" s="16"/>
-      <c r="G59" s="13"/>
-    </row>
-    <row r="60" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B60" s="13"/>
-      <c r="C60" s="13"/>
-      <c r="D60" s="15"/>
-      <c r="E60" s="13"/>
-      <c r="F60" s="16"/>
-      <c r="G60" s="13"/>
-    </row>
-    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B61" s="13"/>
-      <c r="C61" s="13"/>
-      <c r="D61" s="15"/>
-      <c r="E61" s="13"/>
-      <c r="F61" s="16"/>
-      <c r="G61" s="13"/>
-    </row>
-    <row r="62" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B62" s="13"/>
-      <c r="C62" s="13"/>
-      <c r="D62" s="15"/>
-      <c r="E62" s="13"/>
-      <c r="F62" s="16"/>
-      <c r="G62" s="13"/>
-    </row>
-    <row r="63" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B63" s="13"/>
-      <c r="C63" s="13"/>
-      <c r="D63" s="15"/>
-      <c r="E63" s="13"/>
-      <c r="F63" s="16"/>
-      <c r="G63" s="13"/>
-    </row>
-    <row r="64" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B64" s="13"/>
-      <c r="C64" s="13"/>
-      <c r="D64" s="15"/>
-      <c r="E64" s="13"/>
-      <c r="F64" s="16"/>
-      <c r="G64" s="13"/>
-    </row>
-    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B65" s="13"/>
-      <c r="C65" s="13"/>
-      <c r="D65" s="15"/>
-      <c r="E65" s="13"/>
-      <c r="F65" s="16"/>
-      <c r="G65" s="13"/>
-    </row>
-    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D66" s="11"/>
-      <c r="E66" s="11"/>
-      <c r="F66" s="12"/>
-    </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D67" s="11"/>
-      <c r="E67" s="11"/>
-      <c r="F67" s="12"/>
-    </row>
-    <row r="68" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D68" s="11"/>
-      <c r="E68" s="11"/>
-      <c r="F68" s="12"/>
-    </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D69" s="11"/>
-      <c r="E69" s="11"/>
-      <c r="F69" s="12"/>
-    </row>
-    <row r="70" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D70" s="11"/>
-      <c r="E70" s="11"/>
-      <c r="F70" s="12"/>
-    </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D71" s="11"/>
-      <c r="E71" s="11"/>
-      <c r="F71" s="12"/>
-    </row>
-    <row r="72" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D72" s="11"/>
-      <c r="E72" s="11"/>
-      <c r="F72" s="12"/>
-    </row>
-    <row r="73" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D73" s="11"/>
-      <c r="E73" s="11"/>
-      <c r="F73" s="12"/>
-    </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D74" s="11"/>
-      <c r="E74" s="11"/>
-      <c r="F74" s="12"/>
-    </row>
-    <row r="75" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D75" s="11"/>
-      <c r="E75" s="11"/>
-      <c r="F75" s="12"/>
-    </row>
-    <row r="76" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D76" s="11"/>
-      <c r="E76" s="11"/>
-      <c r="F76" s="12"/>
-    </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D77" s="11"/>
-      <c r="E77" s="11"/>
-      <c r="F77" s="12"/>
-    </row>
-    <row r="78" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D78" s="11"/>
-      <c r="E78" s="11"/>
-      <c r="F78" s="12"/>
-    </row>
-    <row r="79" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D79" s="11"/>
-      <c r="E79" s="11"/>
-      <c r="F79" s="12"/>
-    </row>
-    <row r="80" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D80" s="11"/>
-      <c r="E80" s="11"/>
-      <c r="F80" s="12"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="13"/>
+      <c r="G45" s="10"/>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B46" s="10"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="13"/>
+      <c r="G46" s="10"/>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B47" s="21"/>
+      <c r="C47" s="21"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="21"/>
+    </row>
+    <row r="48" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B48" s="21"/>
+      <c r="C48" s="21"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="21"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="21"/>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B49" s="10"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="12"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="10"/>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B50" s="10"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="12"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="13"/>
+      <c r="G50" s="10"/>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="12"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="13"/>
+      <c r="G51" s="10"/>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="12"/>
+      <c r="E52" s="10"/>
+      <c r="F52" s="13"/>
+      <c r="G52" s="10"/>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B53" s="10"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="12"/>
+      <c r="E53" s="10"/>
+      <c r="F53" s="13"/>
+      <c r="G53" s="10"/>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B54" s="10"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="12"/>
+      <c r="E54" s="10"/>
+      <c r="F54" s="13"/>
+      <c r="G54" s="10"/>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B55" s="10"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="12"/>
+      <c r="E55" s="10"/>
+      <c r="F55" s="13"/>
+      <c r="G55" s="10"/>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D56" s="8"/>
+      <c r="E56" s="8"/>
+      <c r="F56" s="9"/>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D57" s="8"/>
+      <c r="E57" s="8"/>
+      <c r="F57" s="9"/>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D58" s="8"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="9"/>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D59" s="8"/>
+      <c r="E59" s="8"/>
+      <c r="F59" s="9"/>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="9"/>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D61" s="8"/>
+      <c r="E61" s="8"/>
+      <c r="F61" s="9"/>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D62" s="8"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="9"/>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D63" s="8"/>
+      <c r="E63" s="8"/>
+      <c r="F63" s="9"/>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D64" s="8"/>
+      <c r="E64" s="8"/>
+      <c r="F64" s="9"/>
+    </row>
+    <row r="65" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D65" s="8"/>
+      <c r="E65" s="8"/>
+      <c r="F65" s="9"/>
+    </row>
+    <row r="66" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D66" s="8"/>
+      <c r="E66" s="8"/>
+      <c r="F66" s="9"/>
+    </row>
+    <row r="67" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D67" s="8"/>
+      <c r="E67" s="8"/>
+      <c r="F67" s="9"/>
+    </row>
+    <row r="68" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D68" s="8"/>
+      <c r="E68" s="8"/>
+      <c r="F68" s="9"/>
+    </row>
+    <row r="69" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D69" s="8"/>
+      <c r="E69" s="8"/>
+      <c r="F69" s="9"/>
+    </row>
+    <row r="70" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="9"/>
+    </row>
+    <row r="71" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D71" s="8"/>
+      <c r="E71" s="8"/>
+      <c r="F71" s="9"/>
+    </row>
+    <row r="72" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D72" s="8"/>
+      <c r="E72" s="8"/>
+      <c r="F72" s="9"/>
+    </row>
+    <row r="73" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D73" s="8"/>
+      <c r="E73" s="8"/>
+      <c r="F73" s="9"/>
+    </row>
+    <row r="74" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D74" s="8"/>
+      <c r="E74" s="8"/>
+      <c r="F74" s="9"/>
+    </row>
+    <row r="75" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D75" s="8"/>
+      <c r="E75" s="8"/>
+      <c r="F75" s="9"/>
+    </row>
+    <row r="76" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D76" s="8"/>
+      <c r="E76" s="8"/>
+      <c r="F76" s="9"/>
+    </row>
+    <row r="77" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D77" s="8"/>
+      <c r="E77" s="8"/>
+      <c r="F77" s="9"/>
+    </row>
+    <row r="78" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D78" s="8"/>
+      <c r="E78" s="8"/>
+      <c r="F78" s="9"/>
+    </row>
+    <row r="79" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D79" s="8"/>
+      <c r="E79" s="8"/>
+      <c r="F79" s="9"/>
+    </row>
+    <row r="80" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D80" s="8"/>
+      <c r="E80" s="8"/>
+      <c r="F80" s="9"/>
     </row>
     <row r="81" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D81" s="11"/>
-      <c r="E81" s="11"/>
-      <c r="F81" s="12"/>
+      <c r="D81" s="8"/>
+      <c r="E81" s="8"/>
+      <c r="F81" s="9"/>
     </row>
     <row r="82" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D82" s="11"/>
-      <c r="E82" s="11"/>
-      <c r="F82" s="12"/>
+      <c r="D82" s="8"/>
+      <c r="E82" s="8"/>
+      <c r="F82" s="9"/>
     </row>
     <row r="83" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D83" s="11"/>
-      <c r="E83" s="11"/>
-      <c r="F83" s="12"/>
+      <c r="D83" s="8"/>
+      <c r="E83" s="8"/>
+      <c r="F83" s="9"/>
     </row>
     <row r="84" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D84" s="11"/>
-      <c r="E84" s="11"/>
-      <c r="F84" s="12"/>
-    </row>
-    <row r="85" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D85" s="11"/>
-      <c r="E85" s="11"/>
-      <c r="F85" s="12"/>
-    </row>
-    <row r="86" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D86" s="11"/>
-      <c r="E86" s="11"/>
-      <c r="F86" s="12"/>
-    </row>
-    <row r="87" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D87" s="11"/>
-      <c r="E87" s="11"/>
-      <c r="F87" s="12"/>
-    </row>
-    <row r="88" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D88" s="11"/>
-      <c r="E88" s="11"/>
-      <c r="F88" s="12"/>
-    </row>
-    <row r="89" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D89" s="11"/>
-      <c r="E89" s="11"/>
-      <c r="F89" s="12"/>
-    </row>
-    <row r="90" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D90" s="11"/>
-      <c r="E90" s="11"/>
-      <c r="F90" s="12"/>
-    </row>
-    <row r="91" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D91" s="11"/>
-      <c r="E91" s="11"/>
-      <c r="F91" s="12"/>
-    </row>
-    <row r="92" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D92" s="11"/>
-      <c r="E92" s="11"/>
-      <c r="F92" s="12"/>
-    </row>
-    <row r="93" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D93" s="11"/>
-      <c r="E93" s="11"/>
-      <c r="F93" s="12"/>
-    </row>
-    <row r="94" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D94" s="11"/>
-      <c r="E94" s="11"/>
-      <c r="F94" s="12"/>
+      <c r="D84" s="8"/>
+      <c r="E84" s="8"/>
+      <c r="F84" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="D1:J1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="6">
-    <mergeCell ref="G57:G58"/>
-    <mergeCell ref="B57:B58"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="D57:D58"/>
-    <mergeCell ref="E57:E58"/>
-    <mergeCell ref="F57:F58"/>
+    <mergeCell ref="G47:G48"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="D47:D48"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="F47:F48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>
@@ -2327,7 +2253,7 @@
       <c r="C10" s="1"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="9" t="s">
         <v>112</v>
       </c>
       <c r="B11" s="2">
@@ -2338,7 +2264,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="9" t="s">
         <v>112</v>
       </c>
       <c r="B12" s="2">
@@ -2349,7 +2275,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="9" t="s">
         <v>112</v>
       </c>
       <c r="B13" s="2">
@@ -2360,7 +2286,7 @@
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="9" t="s">
         <v>112</v>
       </c>
       <c r="B14" s="2">
@@ -2783,38 +2709,38 @@
     <col min="11" max="11" width="87.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="22" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:11" s="19" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="E1" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="F1" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="22" t="s">
+      <c r="G1" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="H1" s="22" t="s">
+      <c r="H1" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="I1" s="22" t="s">
+      <c r="I1" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="J1" s="22" t="s">
+      <c r="J1" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="K1" s="22" t="s">
+      <c r="K1" s="19" t="s">
         <v>39</v>
       </c>
     </row>
@@ -2840,7 +2766,7 @@
       <c r="G2" t="s">
         <v>124</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="H2" s="18" t="s">
         <v>72</v>
       </c>
     </row>
@@ -2890,17 +2816,17 @@
     <col min="4" max="4" width="32" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:4" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="16" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2998,7 +2924,7 @@
       <c r="A8" t="s">
         <v>163</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="9" t="s">
         <v>199</v>
       </c>
     </row>
@@ -3038,10 +2964,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
     </row>
@@ -3049,47 +2975,47 @@
       <c r="A2" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="7" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="9" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="9" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="9" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="9" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3097,87 +3023,87 @@
       <c r="A8" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="7" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="9" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="9" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="9" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="8" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="8" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="14" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="9" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="9" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="9" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="9" t="s">
         <v>95</v>
       </c>
     </row>
@@ -3186,15 +3112,15 @@
       <c r="B19" s="2"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="8" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="9" t="s">
         <v>58</v>
       </c>
       <c r="B21" t="s">
@@ -3202,18 +3128,18 @@
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="7" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="7" t="s">
         <v>128</v>
       </c>
     </row>
@@ -3226,18 +3152,18 @@
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="9" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B26" s="12" t="s">
+      <c r="B26" s="9" t="s">
         <v>136</v>
       </c>
     </row>
@@ -3258,18 +3184,18 @@
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="9" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="9" t="s">
         <v>146</v>
       </c>
     </row>
@@ -3290,50 +3216,50 @@
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="12" t="s">
+      <c r="A37" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B37" s="12" t="s">
+      <c r="B37" s="9" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="12" t="s">
+      <c r="A38" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="B38" s="12" t="s">
+      <c r="B38" s="9" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="12" t="s">
+      <c r="A39" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B39" s="12" t="s">
+      <c r="B39" s="9" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="12" t="s">
+      <c r="A40" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B40" s="12" t="s">
+      <c r="B40" s="9" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="12" t="s">
+      <c r="A41" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B41" s="12" t="s">
+      <c r="B41" s="9" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="12" t="s">
+      <c r="A43" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="B43" s="12" t="s">
+      <c r="B43" s="9" t="s">
         <v>194</v>
       </c>
     </row>

</xml_diff>